<commit_message>
GB6-GB8: grout design-conformance properties, and Occurrence fixes for the retired propertyClass/designProperty elements
designProperty.xml: five new entries (binding_material_content,
water_binding_material_ratio, chloride_content_in_concrete,
differential_settlement, relative_compaction), and all Occurrence bindings
repointed from the now-removed //diggs:DesignConformanceCriterion/diggs:designProperty
to //diggs:parameterName + ancestor::diggs:DesignConformanceCriterion.

properties.xml: the four PerformanceCriterion-scoped Occurrence bindings
(settlement, differential_settlement, settlement_reduction_ratio,
reinforcement_load_fraction) repointed the same way, off the removed
propertyClass element.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1446,60 +1446,160 @@
         <f>IF(ISNA(VLOOKUP(B14,AssociatedElements!B$2:B2952,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B14" s="13" t="n"/>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="13" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>binding_material_content</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Binding material content</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>Mass of binding material (cement plus pozzolanic materials such as fly ash or silica fume) per unit volume of grout/concrete - for example specified with a minimum of 390 kg/m3 under SEC 70-TMSS-03 Table 8B for Very Severe/Severe exposure. A recipe requirement checked against the batch as mixed, not a tested physical property of the cured material - contrast compressive_strength_unconfined (properties.xml), which is.</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F14" s="13" t="n"/>
-      <c r="G14" s="9" t="n"/>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2">
         <f>IF(ISNA(VLOOKUP(B15,AssociatedElements!B$2:B2953,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B15" s="13" t="n"/>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="19" t="n"/>
-      <c r="E15" s="18" t="n"/>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>water_binding_material_ratio</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>Water/binding-material ratio</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Ratio of water mass to binding-material mass (cement plus pozzolanic materials) in a grout/concrete mix - for example specified with a maximum of 0.40 under SEC 70-TMSS-03 Table 8B for a silica-fume mix in Very Severe/Severe exposure. Distinct from the plain water/cement ratio (diggs:DesignGroutMixType/waterCementRatio), which excludes any SCM replacement from the denominator. A recipe requirement checked against the batch as mixed, not a tested physical property of the cured material.</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F15" s="18" t="n"/>
-      <c r="G15" s="9" t="n"/>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2">
         <f>IF(ISNA(VLOOKUP(B16,AssociatedElements!B$2:B2954,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B16" s="13" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="19" t="n"/>
-      <c r="E16" s="18" t="n"/>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>chloride_content_in_concrete</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Chloride content in concrete</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Chloride ion content of a grout/concrete mix, expressed as a percentage of the mix (not of a constituent) - for example limited to a maximum of 0.10% under SEC 70-TMSS-03 Table 8B, fixed across every exposure class regardless of admixture route. DISTINCT FROM properties.xml#chloride_content, which is the chloride content of SOIL OR GROUNDWATER (the exposure condition that selects which Table 8B row applies) - this entry is the durability-relevant quantity in the hardened mix itself, a different subject. A recipe/material requirement checked against the batch as mixed, not an emergent tested behaviour - contrast compressive_strength_unconfined (properties.xml), which is.</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F16" s="18" t="n"/>
-      <c r="G16" s="9" t="n"/>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2">
         <f>IF(ISNA(VLOOKUP(B17,AssociatedElements!B$2:B2955,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="19" t="n"/>
-      <c r="E17" s="18" t="n"/>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>differential_settlement</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>Differential settlement</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Differential settlement between adjacent elements or points, checked against an allowable gradient - the design-side counterpart of properties.xml#differential_settlement, which names the same quantity as MEASURED post-construction. Typically stated per unit length (basis=per unit length, baseLength carrying the reference length) - see diggs:AbstractAcceptanceCriterionType/basis and baseLength.</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F17" s="18" t="n"/>
-      <c r="G17" s="9" t="n"/>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2">
         <f>IF(ISNA(VLOOKUP(B18,AssociatedElements!B$2:B2956,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B18" s="13" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="19" t="n"/>
-      <c r="E18" s="18" t="n"/>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>relative_compaction</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Relative compaction</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>The ratio of the field (as-compacted) dry density of a fill material to a reference maximum dry density (typically from a Proctor compaction test, e.g. ASTM D698/D1557), expressed as a percentage, checked against a specified minimum - for example 95% for a load transfer platform fill. A conformance check on the fill as placed, not a tested physical property of the material itself - distinct from properties.xml#dry_density_max, which is the reference value this ratio is computed against, and from properties.xml#relative_density, an unrelated granular-soil state parameter (Dr).</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F18" s="18" t="n"/>
-      <c r="G18" s="9" t="n"/>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2">
@@ -1776,7 +1876,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1897,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1918,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1939,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1960,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1981,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1872,7 +2002,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1888,7 +2023,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1904,7 +2044,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1920,7 +2065,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1936,7 +2086,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1952,7 +2107,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
         </is>
       </c>
     </row>
@@ -1961,35 +2121,105 @@
         <f>IF(ISNA(VLOOKUP(B14,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B14" s="20" t="n"/>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>binding_material_content</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
         <f>IF(ISNA(VLOOKUP(B15,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B15" s="2" t="n"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>water_binding_material_ratio</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
         <f>IF(ISNA(VLOOKUP(B16,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B16" s="2" t="n"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>chloride_content_in_concrete</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
         <f>IF(ISNA(VLOOKUP(B17,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B17" s="2" t="n"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>differential_settlement</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
         <f>IF(ISNA(VLOOKUP(B18,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B18" s="2" t="n"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>relative_compaction</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19">

</xml_diff>

<commit_message>
EAC6: ValueBindings sheet in the converter; first value bindings in designProperty
- dict_xml_convert.py reads an optional ValueBindings sheet and emits each row as a
  diggs:ValueBinding inside diggs:valueBindings, after occurrences, in row order. Regenerating all
  103 dictionaries with the change reproduces every committed file byte for byte.
- DIGGSDictionaryTemplate.xltx gains the ValueBindings sheet (dropdowns for Method,
  ReferenceSource, ReferenceEvaluation).
- designProperty: 13 bindings on position, verticality, alignment_deviation, diameter, length,
  bearing_stratum_embedment (evidence unit top, design bearing unit, design level),
  water_binding_material_ratio and installation_sequence; new term installation_sequence.
  Additions only (108+/0-).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Lists" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ValueBindings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Lists" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -128,6 +129,9 @@
       <sz val="8"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -191,7 +195,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -243,6 +247,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1606,12 +1611,32 @@
         <f>IF(ISNA(VLOOKUP(B19,AssociatedElements!B$2:B2957,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B19" s="13" t="n"/>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="19" t="n"/>
-      <c r="E19" s="18" t="n"/>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>installation_sequence</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Installation sequence</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Whether an element was installed in its designed order relative to its design neighbours - after its nearest built design predecessor and before its nearest built design successor in the governing design's installation sequence. Evaluated as true or false (operator eq, limit true). Comparing an as-built installation number with a design sequence number directly is not meaningful: one element installed out of order shifts the number of every element after it.</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F19" s="18" t="n"/>
-      <c r="G19" s="9" t="n"/>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2">
@@ -2226,7 +2251,21 @@
         <f>IF(ISNA(VLOOKUP(B19,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B19" s="20" t="n"/>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>installation_sequence</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -2436,6 +2475,589 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="B1" s="21" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C1" s="21" t="inlineStr">
+        <is>
+          <t>SubjectElement</t>
+        </is>
+      </c>
+      <c r="D1" s="21" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="E1" s="21" t="inlineStr">
+        <is>
+          <t>RealizedValueXpath</t>
+        </is>
+      </c>
+      <c r="F1" s="21" t="inlineStr">
+        <is>
+          <t>ReferenceValueXpath</t>
+        </is>
+      </c>
+      <c r="G1" s="21" t="inlineStr">
+        <is>
+          <t>ReferenceSource</t>
+        </is>
+      </c>
+      <c r="H1" s="21" t="inlineStr">
+        <is>
+          <t>ReferenceEvaluation</t>
+        </is>
+      </c>
+      <c r="I1" s="21" t="inlineStr">
+        <is>
+          <t>NormalizeByXpath</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>IF(ISNA(VLOOKUP(B2,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>water_binding_material_ratio</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>diggs:GroutBatch</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>diggs:waterCementRatioOfMix</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <f>IF(ISNA(VLOOKUP(B3,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>horizontal_offset</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>diggs:referencePoint</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>diggs:scope/diggs:SFDesignScope/diggs:targetPosition</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <f>IF(ISNA(VLOOKUP(B4,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>horizontal_offset</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>diggs:referencePoint</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>diggs:scope/diggs:SFDesignScope/diggs:plannedPositions</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <f>IF(ISNA(VLOOKUP(B5,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>verticality</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>diggs:alignmentDeviation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <f>IF(ISNA(VLOOKUP(B6,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>alignment_deviation</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>diggs:alignmentDeviation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <f>IF(ISNA(VLOOKUP(B7,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>alignment_deviation</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>angular_difference</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>diggs:plunge</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>diggs:designPlunge</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <f>IF(ISNA(VLOOKUP(B8,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>diameter</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>diggs:columnDiameter</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>diggs:columnDiameter</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <f>IF(ISNA(VLOOKUP(B9,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>diggs:columnLength</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>diggs:columnLength</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <f>IF(ISNA(VLOOKUP(B10,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>bearing_stratum_embedment</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>reverse_difference</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>number(tokenize(normalize-space(diggs:centerLine//gml:posList),'\s+')[last()])</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>diggs:location</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>volume_top</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>diggs:columnDiameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <f>IF(ISNA(VLOOKUP(B11,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>bearing_stratum_embedment</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>reverse_difference</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>number(tokenize(normalize-space(diggs:centerLine//gml:posList),'\s+')[last()])</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>diggs:deref(diggs:bearingUnitRef)/diggs:location</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>volume_top</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>diggs:columnDiameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <f>IF(ISNA(VLOOKUP(B12,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>bearing_stratum_embedment</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>reverse_difference</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>number(tokenize(normalize-space(diggs:centerLine//gml:posList),'\s+')[last()])</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>(diggs:geoUnitDesignQuantity//diggs:bearingStratumLevel//gml:pos)[1]</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>diggs:columnDiameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <f>IF(ISNA(VLOOKUP(B13,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>installation_sequence</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>diggs:RIColumn</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>sequence_between</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>diggs:installationSequenceNumber</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <f>IF(ISNA(VLOOKUP(B14,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>installation_sequence</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>diggs:RIColumn</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>sequence_between</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>diggs:whenConstructed//diggs:start</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <f>IF(ISNA(VLOOKUP(B15,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <f>IF(ISNA(VLOOKUP(B16,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <f>IF(ISNA(VLOOKUP(B17,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <f>IF(ISNA(VLOOKUP(B18,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <f>IF(ISNA(VLOOKUP(B19,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <f>IF(ISNA(VLOOKUP(B20,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <f>IF(ISNA(VLOOKUP(B21,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <f>IF(ISNA(VLOOKUP(B22,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <f>IF(ISNA(VLOOKUP(B23,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <f>IF(ISNA(VLOOKUP(B24,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <f>IF(ISNA(VLOOKUP(B25,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <f>IF(ISNA(VLOOKUP(B26,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <f>IF(ISNA(VLOOKUP(B27,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <f>IF(ISNA(VLOOKUP(B28,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <f>IF(ISNA(VLOOKUP(B29,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <f>IF(ISNA(VLOOKUP(B30,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <f>IF(ISNA(VLOOKUP(B31,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="D2:D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"direct,horizontal_offset,difference,reverse_difference,angular_difference,containment,sequence_between,value_at,rate,rate_per_log_cycle,within_envelope,frequency"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"design,evidence"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"value,vertical_intersection,volume_top,volume_base"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E188"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>

</xml_diff>

<commit_message>
EAC7b: value binding for binding_material_content (GroutBatch/bindingMaterialContent)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9200" yWindow="3280" windowWidth="39400" windowHeight="24940" tabRatio="500" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ValueBindings" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Lists" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValueBindings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1000,7 +1000,7 @@
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -2938,6 +2938,26 @@
       <c r="A15">
         <f>IF(ISNA(VLOOKUP(B15,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>binding_material_content</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>diggs:GroutBatch</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>diggs:bindingMaterialContent</t>
+        </is>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
EAC7c: value binding for chloride_content_in_concrete (GroutBatch/chlorideContentOfMix)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -2965,6 +2965,26 @@
         <f>IF(ISNA(VLOOKUP(B16,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>chloride_content_in_concrete</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>diggs:GroutBatch</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>diggs:chlorideContentOfMix</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17">

</xml_diff>

<commit_message>
EAC7d: designProperty water_soluble/acid_soluble_chloride_content_in_concrete with value bindings (replaces chloride_content_in_concrete)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1517,17 +1517,17 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>chloride_content_in_concrete</t>
+          <t>water_soluble_chloride_content_in_concrete</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>Chloride content in concrete</t>
+          <t>Water-soluble chloride content in concrete</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Chloride ion content of a grout/concrete mix, expressed as a percentage of the mix (not of a constituent) - for example limited to a maximum of 0.10% under SEC 70-TMSS-03 Table 8B, fixed across every exposure class regardless of admixture route. DISTINCT FROM properties.xml#chloride_content, which is the chloride content of SOIL OR GROUNDWATER (the exposure condition that selects which Table 8B row applies) - this entry is the durability-relevant quantity in the hardened mix itself, a different subject. A recipe/material requirement checked against the batch as mixed, not an emergent tested behaviour - contrast compressive_strength_unconfined (properties.xml), which is.</t>
+          <t>Water-soluble chloride ion (Cl-) content of hardened grout or concrete, expressed as a mass fraction of the cement (for example %) - for example limited to a maximum of 0.10% by mass of cement under SEC 70-TMSS-03. The chloride that dissolves in water under the conditions of the test method (ASTM C1218/C1218M); a different quantity from acid-soluble chloride (acid_soluble_chloride_content_in_concrete), which a specification may limit separately. DISTINCT FROM properties.xml#chloride_content, which is the chloride content of SOIL OR GROUNDWATER (the exposure condition that selects the requirements) - this entry is the durability-relevant quantity in the concrete itself, a different subject. Compliance is shown by testing; a mix design does not by itself establish it.</t>
         </is>
       </c>
       <c r="E16" s="18" t="inlineStr">
@@ -1643,12 +1643,32 @@
         <f>IF(ISNA(VLOOKUP(B20,AssociatedElements!B$2:B2958,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="18" t="n"/>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>acid_soluble_chloride_content_in_concrete</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Acid-soluble chloride content in concrete</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Acid-soluble chloride ion (Cl-) content of hardened grout or concrete, expressed as a mass fraction of the cement (for example %). The chloride that dissolves in acid under the conditions of the test method (ASTM C1152/C1152M), which in most concretes approximates the total chloride; a different quantity from water-soluble chloride (water_soluble_chloride_content_in_concrete), which a specification may limit separately and at a different value. DISTINCT FROM properties.xml#chloride_content, which is the chloride content of SOIL OR GROUNDWATER. Compliance is shown by testing; a mix design does not by itself establish it.</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F20" s="18" t="n"/>
-      <c r="G20" s="9" t="n"/>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2">
@@ -2190,7 +2210,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>chloride_content_in_concrete</t>
+          <t>water_soluble_chloride_content_in_concrete</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2272,7 +2292,21 @@
         <f>IF(ISNA(VLOOKUP(B20,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B20" s="20" t="n"/>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>acid_soluble_chloride_content_in_concrete</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -2967,7 +3001,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chloride_content_in_concrete</t>
+          <t>water_soluble_chloride_content_in_concrete</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2982,7 +3016,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>diggs:chlorideContentOfMix</t>
+          <t>diggs:waterSolubleChlorideContent</t>
         </is>
       </c>
     </row>
@@ -2990,6 +3024,26 @@
       <c r="A17">
         <f>IF(ISNA(VLOOKUP(B17,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>acid_soluble_chloride_content_in_concrete</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>diggs:GroutBatch</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>diggs:acidSolubleChlorideContent</t>
+        </is>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
EAC7e: designProperty sampling_frequency; dictionary description covers compositional and procedural properties
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -990,7 +990,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Codes naming the design property a diggs:DesignConformanceCriterion governs - a geometric or constructional property measured against its design intent, as opposed to a diggs:PerformanceCriterion's measured physical property. Used for the value of the designProperty property of diggs:DesignConformanceCriterionType. The intended value set is stated directly in the schema's own documentation for this element.</t>
+          <t>Codes naming the design property a diggs:DesignConformanceCriterion governs - a geometric, constructional, compositional or procedural property checked against what the design or specification requires, as opposed to a diggs:PerformanceCriterion's measured physical property. Used for the value of the designProperty property of diggs:DesignConformanceCriterionType. The intended value set is stated directly in the schema's own documentation for this element.</t>
         </is>
       </c>
     </row>
@@ -1675,12 +1675,32 @@
         <f>IF(ISNA(VLOOKUP(B21,AssociatedElements!B$2:B2959,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B21" s="13" t="n"/>
-      <c r="C21" s="18" t="n"/>
-      <c r="D21" s="19" t="n"/>
-      <c r="E21" s="18" t="n"/>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>sampling_frequency</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Acceptance sampling frequency</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Number of acceptance samplings taken per unit volume of material placed - for example a minimum of 1 sampling per 100 m3 of concrete for compressive strength testing. A requirement on how much testing is done, not on a measured property of the material: it is met by counting the distinct samplings behind the test results, so results reported only as an average cannot show it was met.</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F21" s="18" t="n"/>
-      <c r="G21" s="9" t="n"/>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2">
@@ -2313,7 +2333,21 @@
         <f>IF(ISNA(VLOOKUP(B21,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B21" s="20" t="n"/>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>sampling_frequency</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22">

</xml_diff>

<commit_message>
LTS1: relative_compaction dataType double/dimensionless; relative_density bound to DesignConformanceCriterion; evidenceCondition fines_content
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1591,15 +1591,19 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>The ratio of the field (as-compacted) dry density of a fill material to a reference maximum dry density (typically from a Proctor compaction test, e.g. ASTM D698/D1557), expressed as a percentage, checked against a specified minimum - for example 95% for a load transfer platform fill. A conformance check on the fill as placed, not a tested physical property of the material itself - distinct from properties.xml#dry_density_max, which is the reference value this ratio is computed against, and from properties.xml#relative_density, an unrelated granular-soil state parameter (Dr).</t>
+          <t>The ratio of the field (as-compacted) dry density of a fill material to a reference maximum dry density (typically from a Proctor compaction test, e.g. ASTM D698/D1557), expressed as a percentage, checked against a specified minimum or range - for example 95% for a load transfer platform fill. A conformance check on the fill as placed, not a tested physical property of the material itself - distinct from properties.xml#dry_density_max, which is the reference value this ratio is computed against, and from properties.xml#relative_density, an unrelated granular-soil state parameter (Dr).</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="n"/>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
           <t>DIGGS</t>

</xml_diff>

<commit_message>
RICS1: designProperty radial/easting/northing_position_deviation, length_deviation, penetration_over_interval, discharge_time; evidenceCondition interval_duration
Six DesignConformanceCriterion design properties for rigid inclusion column acceptance (position tolerance in radial and per-axis forms,
length against design, refusal penetration over an interval, grout/concrete discharge time) and the interval_duration evidence condition
that states the interval. Workbook-first, regenerated with dict_xml_convert.py --only; additions only (96 + 16 lines, 0 deletions).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1711,66 +1711,216 @@
         <f>IF(ISNA(VLOOKUP(B22,AssociatedElements!B$2:B2960,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="19" t="n"/>
-      <c r="E22" s="18" t="n"/>
-      <c r="F22" s="18" t="n"/>
-      <c r="G22" s="9" t="n"/>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>radial_position_deviation</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Radial position deviation</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>The plan (horizontal) distance between the as-built position of the element and its designed position - the radial form of a position tolerance. Use easting_position_deviation and northing_position_deviation where a tolerance is stated per axis.</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2">
         <f>IF(ISNA(VLOOKUP(B23,AssociatedElements!B$2:B2961,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B23" s="13" t="n"/>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="19" t="n"/>
-      <c r="E23" s="18" t="n"/>
-      <c r="F23" s="18" t="n"/>
-      <c r="G23" s="9" t="n"/>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>easting_position_deviation</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>Easting position deviation</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>The signed offset, along the easting axis of the project horizontal CRS, of the as-built position of the element from its designed position (positive towards increasing easting). The per-axis form of a position tolerance; see radial_position_deviation for the radial form.</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2">
         <f>IF(ISNA(VLOOKUP(B24,AssociatedElements!B$2:B2962,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="D24" s="16" t="n"/>
-      <c r="G24" s="9" t="n"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>northing_position_deviation</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Northing position deviation</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>The signed offset, along the northing axis of the project horizontal CRS, of the as-built position of the element from its designed position (positive towards increasing northing). The per-axis form of a position tolerance; see radial_position_deviation for the radial form.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2">
         <f>IF(ISNA(VLOOKUP(B25,AssociatedElements!B$2:B2963,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B25" s="13" t="n"/>
-      <c r="C25" s="13" t="n"/>
-      <c r="E25" s="13" t="n"/>
-      <c r="F25" s="13" t="n"/>
-      <c r="G25" s="9" t="n"/>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>length_deviation</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Length deviation</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>The as-built length of the element minus its designed length, signed: negative where the element is shorter than designed. Use it where a requirement limits the shortfall or excess against design; length states the absolute as-built length.</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2">
         <f>IF(ISNA(VLOOKUP(B26,AssociatedElements!B$2:B2964,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B26" s="13" t="n"/>
-      <c r="C26" s="13" t="n"/>
-      <c r="E26" s="13" t="n"/>
-      <c r="F26" s="13" t="n"/>
-      <c r="G26" s="9" t="n"/>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>penetration_over_interval</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Penetration over an interval</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>The distance the installation tool advances into the ground over a stated interval of time - for example less than 50 mm over two consecutive minutes as a drilling refusal rule. The interval is stated by an evidenceCondition (interval_duration) on the criterion. Distinct from penetration_rate, which is the same advance expressed per unit time.</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2">
         <f>IF(ISNA(VLOOKUP(B27,AssociatedElements!B$2:B2965,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B27" s="13" t="n"/>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13" t="n"/>
-      <c r="G27" s="9" t="n"/>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>discharge_time</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Discharge time</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>The time elapsed from the introduction of mixing water to the end of discharge of the mix at the point of placement - a limit on how long a grout or concrete batch may take to be placed.</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2">
@@ -2358,42 +2508,126 @@
         <f>IF(ISNA(VLOOKUP(B22,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B22" s="20" t="n"/>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>radial_position_deviation</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
         <f>IF(ISNA(VLOOKUP(B23,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B23" s="20" t="n"/>
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>easting_position_deviation</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
         <f>IF(ISNA(VLOOKUP(B24,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B24" s="2" t="n"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>northing_position_deviation</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
         <f>IF(ISNA(VLOOKUP(B25,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B25" s="2" t="n"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>length_deviation</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
         <f>IF(ISNA(VLOOKUP(B26,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B26" s="2" t="n"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>penetration_over_interval</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
         <f>IF(ISNA(VLOOKUP(B27,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B27" s="13" t="n"/>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>discharge_time</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28">

</xml_diff>

<commit_message>
RICS1: designProperty - remove radial_position_deviation; bind easting/northing deviations; length is absolute, length_deviation carries the difference
- position stays as the radial plan distance (its two horizontal_offset bindings unchanged); radial_position_deviation removed as redundant.
- easting_position_deviation / northing_position_deviation: difference bindings on the coordinates of the column referencePoint and the design targetPosition;
  descriptions state that both positions are in the same CRS.
- length: description and binding made absolute (direct on columnLength); the as-built-minus-design difference binding moves to length_deviation.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1092,7 +1092,7 @@
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>The as-built plan position of the element, measured against its designed position.</t>
+          <t>The plan (horizontal) distance between the as-built position of the element (its reference point) and its designed position - the radial form of a position tolerance. Use easting_position_deviation and northing_position_deviation where a tolerance is stated per axis.</t>
         </is>
       </c>
       <c r="E2" s="13" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>The as-built length of the element, measured against its designed length.</t>
+          <t>The as-built length of the element. Use length_deviation where a requirement is stated against the designed length.</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -1713,17 +1713,17 @@
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>radial_position_deviation</t>
+          <t>easting_position_deviation</t>
         </is>
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>Radial position deviation</t>
+          <t>Easting position deviation</t>
         </is>
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>The plan (horizontal) distance between the as-built position of the element and its designed position - the radial form of a position tolerance. Use easting_position_deviation and northing_position_deviation where a tolerance is stated per axis.</t>
+          <t>The signed offset, along the easting axis of the project horizontal CRS, of the as-built position of the element from its designed position (positive towards increasing easting). The per-axis form of a position tolerance; the as-built and designed positions must be stated in the same CRS, and the axes are taken from its definition; see radial_position_deviation for the radial form.</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
@@ -1749,17 +1749,17 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>easting_position_deviation</t>
+          <t>northing_position_deviation</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Easting position deviation</t>
+          <t>Northing position deviation</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>The signed offset, along the easting axis of the project horizontal CRS, of the as-built position of the element from its designed position (positive towards increasing easting). The per-axis form of a position tolerance; see radial_position_deviation for the radial form.</t>
+          <t>The signed offset, along the northing axis of the project horizontal CRS, of the as-built position of the element from its designed position (positive towards increasing northing). The per-axis form of a position tolerance; the as-built and designed positions must be stated in the same CRS, and the axes are taken from its definition; see radial_position_deviation for the radial form.</t>
         </is>
       </c>
       <c r="E23" s="18" t="inlineStr">
@@ -1785,17 +1785,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>northing_position_deviation</t>
+          <t>length_deviation</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Northing position deviation</t>
+          <t>Length deviation</t>
         </is>
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>The signed offset, along the northing axis of the project horizontal CRS, of the as-built position of the element from its designed position (positive towards increasing northing). The per-axis form of a position tolerance; see radial_position_deviation for the radial form.</t>
+          <t>The as-built length of the element minus its designed length, signed: negative where the element is shorter than designed. Use it where a requirement limits the shortfall or excess against design; length states the absolute as-built length.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1821,17 +1821,17 @@
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>length_deviation</t>
+          <t>penetration_over_interval</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>Length deviation</t>
+          <t>Penetration over an interval</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>The as-built length of the element minus its designed length, signed: negative where the element is shorter than designed. Use it where a requirement limits the shortfall or excess against design; length states the absolute as-built length.</t>
+          <t>The distance the installation tool advances into the ground over a stated interval of time - for example less than 50 mm over two consecutive minutes as a drilling refusal rule. The interval is stated by an evidenceCondition (interval_duration) on the criterion. Distinct from penetration_rate, which is the same advance expressed per unit time.</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -1857,17 +1857,17 @@
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>penetration_over_interval</t>
+          <t>discharge_time</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Penetration over an interval</t>
+          <t>Discharge time</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>The distance the installation tool advances into the ground over a stated interval of time - for example less than 50 mm over two consecutive minutes as a drilling refusal rule. The interval is stated by an evidenceCondition (interval_duration) on the criterion. Distinct from penetration_rate, which is the same advance expressed per unit time.</t>
+          <t>The time elapsed from the introduction of mixing water to the end of discharge of the mix at the point of placement - a limit on how long a grout or concrete batch may take to be placed.</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="F26" s="13" t="inlineStr">
         <is>
-          <t>length</t>
+          <t>time</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
@@ -1891,36 +1891,12 @@
         <f>IF(ISNA(VLOOKUP(B27,AssociatedElements!B$2:B2965,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>discharge_time</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>Discharge time</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="inlineStr">
-        <is>
-          <t>The time elapsed from the introduction of mixing water to the end of discharge of the mix at the point of placement - a limit on how long a grout or concrete batch may take to be placed.</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
-          <t>double</t>
-        </is>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
-        <is>
-          <t>time</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>DIGGS</t>
-        </is>
-      </c>
+      <c r="B27" s="13" t="n"/>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="15" t="n"/>
+      <c r="E27" s="13" t="n"/>
+      <c r="F27" s="13" t="n"/>
+      <c r="G27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2">
@@ -2510,7 +2486,7 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>radial_position_deviation</t>
+          <t>easting_position_deviation</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2531,7 +2507,7 @@
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>easting_position_deviation</t>
+          <t>northing_position_deviation</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2552,7 +2528,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>northing_position_deviation</t>
+          <t>length_deviation</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2573,7 +2549,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>length_deviation</t>
+          <t>penetration_over_interval</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2594,7 +2570,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>penetration_over_interval</t>
+          <t>discharge_time</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2613,21 +2589,7 @@
         <f>IF(ISNA(VLOOKUP(B27,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>discharge_time</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>//diggs:parameterName</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>ancestor::diggs:DesignConformanceCriterion</t>
-        </is>
-      </c>
+      <c r="B27" s="13" t="n"/>
     </row>
     <row r="28">
       <c r="A28">
@@ -3046,22 +3008,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>difference</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>diggs:columnLength</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>diggs:columnLength</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>design</t>
         </is>
       </c>
     </row>
@@ -3323,17 +3275,92 @@
         <f>IF(ISNA(VLOOKUP(B18,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>easting_position_deviation</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>number(tokenize(normalize-space(diggs:referencePoint//gml:pos),'\s+')[1])</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>number(tokenize(normalize-space(diggs:scope/diggs:SFDesignScope/diggs:targetPosition//gml:pos),'\s+')[1])</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
         <f>IF(ISNA(VLOOKUP(B19,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>northing_position_deviation</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>number(tokenize(normalize-space(diggs:referencePoint//gml:pos),'\s+')[2])</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>number(tokenize(normalize-space(diggs:scope/diggs:SFDesignScope/diggs:targetPosition//gml:pos),'\s+')[2])</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
         <f>IF(ISNA(VLOOKUP(B20,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>length_deviation</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>diggs:columnLength</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>diggs:columnLength</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
RICS1: easting/northing_position_deviation - second binding against the planned grid node
Binding 1 (difference) compares the referencePoint coordinate with the design targetPosition. Binding 2 (direct) computes the planned node from
the governing design's RectifiedGrid (found up the basedOnRef chain) at the subject's realizesGridIndex and returns the as-built coordinate minus
the node coordinate; written as direct because the grid index belongs to the subject while a reference path is evaluated against the design.
Tested with Saxon-JS xsl:evaluate on all 1099 RIColumns in SaudiTestCase.xml: each resolves through exactly one binding (1050 grid, 49 target)
and agrees exactly with an independent calculation.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -3368,11 +3368,41 @@
         <f>IF(ISNA(VLOOKUP(B21,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>easting_position_deviation</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>if (exists(diggs:realizesGridIndex)) then (let $d := ($design, diggs:deref($design/diggs:basedOnRef), diggs:deref(diggs:deref($design/diggs:basedOnRef)/diggs:basedOnRef)), $g := ($d/diggs:scope/diggs:SFDesignScope/diggs:plannedPositions//diggs:RectifiedGrid)[1] return if (exists($g)) then (let $i := number(tokenize(normalize-space(diggs:realizesGridIndex),'\s+')[1]), $j := number(tokenize(normalize-space(diggs:realizesGridIndex),'\s+')[2]), $o := tokenize(normalize-space($g/diggs:origin//gml:pos),'\s+'), $a := tokenize(normalize-space($g/diggs:offsetVector[1]),'\s+'), $b := tokenize(normalize-space($g/diggs:offsetVector[2]),'\s+') return number(tokenize(normalize-space(diggs:referencePoint//gml:pos),'\s+')[1]) - (number($o[1]) + $i*number($a[1]) + $j*number($b[1]))) else ()) else ()</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
         <f>IF(ISNA(VLOOKUP(B22,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>northing_position_deviation</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>if (exists(diggs:realizesGridIndex)) then (let $d := ($design, diggs:deref($design/diggs:basedOnRef), diggs:deref(diggs:deref($design/diggs:basedOnRef)/diggs:basedOnRef)), $g := ($d/diggs:scope/diggs:SFDesignScope/diggs:plannedPositions//diggs:RectifiedGrid)[1] return if (exists($g)) then (let $i := number(tokenize(normalize-space(diggs:realizesGridIndex),'\s+')[1]), $j := number(tokenize(normalize-space(diggs:realizesGridIndex),'\s+')[2]), $o := tokenize(normalize-space($g/diggs:origin//gml:pos),'\s+'), $a := tokenize(normalize-space($g/diggs:offsetVector[1]),'\s+'), $b := tokenize(normalize-space($g/diggs:offsetVector[2]),'\s+') return number(tokenize(normalize-space(diggs:referencePoint//gml:pos),'\s+')[2]) - (number($o[2]) + $i*number($a[2]) + $j*number($b[2]))) else ()) else ()</t>
+        </is>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
RICS1: position - second binding is the radial distance to the planned grid node
Replaces the horizontal_offset binding against plannedPositions (a grid, not a position, and only on the cited design) with a direct expression:
the planned node from the governing design's RectifiedGrid (up the basedOnRef chain) at the subject's realizesGridIndex, and the plan distance
from the referencePoint to it. Tested on all 1099 RIColumns in SaudiTestCase.xml (1050 resolve, 49 fall to the targetPosition binding).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -2873,22 +2873,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>horizontal_offset</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>diggs:referencePoint</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>diggs:scope/diggs:SFDesignScope/diggs:plannedPositions</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>design</t>
+          <t>if (exists(diggs:realizesGridIndex)) then (let $d := ($design, diggs:deref($design/diggs:basedOnRef), diggs:deref(diggs:deref($design/diggs:basedOnRef)/diggs:basedOnRef)), $g := ($d/diggs:scope/diggs:SFDesignScope/diggs:plannedPositions//diggs:RectifiedGrid)[1] return if (exists($g)) then (let $i := number(tokenize(normalize-space(diggs:realizesGridIndex),'\s+')[1]), $j := number(tokenize(normalize-space(diggs:realizesGridIndex),'\s+')[2]), $o := tokenize(normalize-space($g/diggs:origin//gml:pos),'\s+'), $a := tokenize(normalize-space($g/diggs:offsetVector[1]),'\s+'), $b := tokenize(normalize-space($g/diggs:offsetVector[2]),'\s+'), $p := tokenize(normalize-space(diggs:referencePoint//gml:pos),'\s+'), $dx := number($p[1]) - (number($o[1]) + $i*number($a[1]) + $j*number($b[1])), $dy := number($p[2]) - (number($o[2]) + $i*number($a[2]) + $j*number($b[2])) return math:sqrt($dx*$dx + $dy*$dy)) else ()) else ()</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RICS1: designProperty - diameter is absolute (direct binding), diameter_deviation carries the design difference; easting/northing descriptions point at position
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1156,7 +1156,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>The as-built diameter of the element, measured against its designed diameter.</t>
+          <t>The as-built diameter of the element. Use diameter_deviation where a requirement is stated against the designed diameter.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>The signed offset, along the easting axis of the project horizontal CRS, of the as-built position of the element from its designed position (positive towards increasing easting). The per-axis form of a position tolerance; the as-built and designed positions must be stated in the same CRS, and the axes are taken from its definition; see radial_position_deviation for the radial form.</t>
+          <t>The signed offset, along the easting axis of the project horizontal CRS, of the as-built position of the element from its designed position (positive towards increasing easting). The per-axis form of a position tolerance; the as-built and designed positions must be stated in the same CRS, and the axes are taken from its definition; see position for the radial form.</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>The signed offset, along the northing axis of the project horizontal CRS, of the as-built position of the element from its designed position (positive towards increasing northing). The per-axis form of a position tolerance; the as-built and designed positions must be stated in the same CRS, and the axes are taken from its definition; see radial_position_deviation for the radial form.</t>
+          <t>The signed offset, along the northing axis of the project horizontal CRS, of the as-built position of the element from its designed position (positive towards increasing northing). The per-axis form of a position tolerance; the as-built and designed positions must be stated in the same CRS, and the axes are taken from its definition; see position for the radial form.</t>
         </is>
       </c>
       <c r="E23" s="18" t="inlineStr">
@@ -1891,12 +1891,36 @@
         <f>IF(ISNA(VLOOKUP(B27,AssociatedElements!B$2:B2965,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B27" s="13" t="n"/>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13" t="n"/>
-      <c r="G27" s="9" t="n"/>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>diameter_deviation</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Diameter deviation</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>The as-built diameter of the element minus its designed diameter, signed: negative where the element is narrower than designed. Use it where a requirement limits the deviation from the designed diameter; diameter states the absolute as-built diameter.</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2">
@@ -2589,7 +2613,21 @@
         <f>IF(ISNA(VLOOKUP(B27,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B27" s="13" t="n"/>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>diameter_deviation</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -2967,22 +3005,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>difference</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>diggs:columnDiameter</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>diggs:columnDiameter</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>design</t>
         </is>
       </c>
     </row>
@@ -3399,6 +3427,31 @@
       <c r="A23">
         <f>IF(ISNA(VLOOKUP(B23,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>diameter_deviation</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>diggs:columnDiameter</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>diggs:columnDiameter</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
RCON1: designProperty - value bindings for discharge_time (installation record end, else whenConstructed end, less batch sampling start) and sampling_frequency (distinct specimen creation times, else casting date from test date and age, per batch volume)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1691,7 +1691,7 @@
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Number of acceptance samplings taken per unit volume of material placed - for example a minimum of 1 sampling per 100 m3 of concrete for compressive strength testing. A requirement on how much testing is done, not on a measured property of the material: it is met by counting the distinct samplings behind the test results, so results reported only as an average cannot show it was met.</t>
+          <t>Number of acceptance samplings taken per unit volume of material placed - for example a minimum of 1 sampling per 100 m3 of concrete for compressive strength testing. A requirement on how much testing is done, not on a measured property of the material: it is met by counting the distinct samplings behind the test results, so results reported only as an average cannot show it was met. A sampling is identified by the creation time of its specimens (extractionTime) or, where that is not recorded, by the casting date derived from the test date and the specimen age at test in days; specimens cast from one sampling share that time, so distinct creation times count samplings. Evaluated per batch against its total batch volume.</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>The time elapsed from the introduction of mixing water to the end of discharge of the mix at the point of placement - a limit on how long a grout or concrete batch may take to be placed.</t>
+          <t>The time elapsed from the introduction of mixing water to the end of discharge of the mix at the point of placement - a limit on how long a grout or concrete batch may take to be placed. Evaluated on the element that received the batch: the end of its installation record where one exists, otherwise the end of its whenConstructed interval, less the start of the batch's sampling (mixing) activity. The two times must be recorded to a resolution at least as fine as the unit of the limit (hours need a time of day; days need only a date); otherwise the value is not evaluable.</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -3459,23 +3459,133 @@
         <f>IF(ISNA(VLOOKUP(B24,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>discharge_time</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>diggs:RIColumn</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>let $id := concat('#', @gml:id) return sort(root(.)//diggs:RIColumnConstruction[diggs:samplingFeatureRef/@xlink:href = $id]/diggs:installationRecord//diggs:timeDomain//(gml:timePosition | gml:endPosition | diggs:end))[last()]</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>(diggs:samplingDate | diggs:deref(diggs:samplingActivityRef)/diggs:samplingDate)/diggs:TimeInterval/diggs:start</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
         <f>IF(ISNA(VLOOKUP(B25,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>discharge_time</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>diggs:RIColumn</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>diggs:whenConstructed//diggs:end</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>(diggs:samplingDate | diggs:deref(diggs:samplingActivityRef)/diggs:samplingDate)/diggs:TimeInterval/diggs:start</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
         <f>IF(ISNA(VLOOKUP(B26,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>sampling_frequency</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>diggs:GroutBatch</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>frequency</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>distinct-values($evidence//diggs:GroutSpecimen/diggs:extractionTime/normalize-space(.))</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>diggs:totalBatchVolume</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
         <f>IF(ISNA(VLOOKUP(B27,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>sampling_frequency</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>diggs:GroutBatch</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>frequency</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>distinct-values(for $s in $evidence//diggs:GroutSpecimen[diggs:ageAtTest[@uom='d']] return string(xs:date(substring(string($s/ancestor::diggs:MaterialTest/diggs:samplingTime//gml:timePosition), 1, 10)) - xs:dayTimeDuration(concat('P', $s/diggs:ageAtTest, 'D'))))</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>diggs:totalBatchVolume</t>
+        </is>
       </c>
     </row>
     <row r="28">

</xml_diff>

<commit_message>
RCON1: penetration_over_interval - change_over_window binding on the installation record depth series
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1831,7 +1831,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>The distance the installation tool advances into the ground over a stated interval of time - for example less than 50 mm over two consecutive minutes as a drilling refusal rule. The interval is stated by an evidenceCondition (interval_duration) on the criterion. Distinct from penetration_rate, which is the same advance expressed per unit time.</t>
+          <t>The distance the installation tool advances into the ground over a stated interval of time - for example less than 50 mm over two consecutive minutes as a drilling refusal rule. The interval is stated by an evidenceCondition (interval_duration) on the criterion. Distinct from penetration_rate, which is the same advance expressed per unit time. Evaluated on the installation record: the depth gained over the window of that duration that ends when the tool first reaches its maximum depth, so a refusal rule judges the last push before termination and not the pause at total depth. Depth is positive downward.</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -3592,6 +3592,36 @@
       <c r="A28">
         <f>IF(ISNA(VLOOKUP(B28,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>penetration_over_interval</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>diggs:RIColumn</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>change_over_window</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>diggs:series(($evidence/descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth')</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>let $s := diggs:series((descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth'), $m := max($s ! ?2) return ($s[?2 = $m])[1]?1</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
RCON1: discharge_time - installation record end from a time-interval-list domain (activity start plus last elapsed time), ahead of the instant-domain and whenConstructed bindings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1867,7 +1867,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>The time elapsed from the introduction of mixing water to the end of discharge of the mix at the point of placement - a limit on how long a grout or concrete batch may take to be placed. Evaluated on the element that received the batch: the end of its installation record where one exists, otherwise the end of its whenConstructed interval, less the start of the batch's sampling (mixing) activity. The two times must be recorded to a resolution at least as fine as the unit of the limit (hours need a time of day; days need only a date); otherwise the value is not evaluable.</t>
+          <t>The time elapsed from the introduction of mixing water to the end of discharge of the mix at the point of placement - a limit on how long a grout or concrete batch may take to be placed. Evaluated on the element that received the batch: the end of its installation record where one exists (the activity start plus the last elapsed time of a time-interval-list domain, or the last time of an instant domain), otherwise the end of its whenConstructed interval, less the start of the batch's sampling (mixing) activity. The two times must be recorded to a resolution at least as fine as the unit of the limit (hours need a time of day; days need only a date); otherwise the value is not evaluable.</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>let $id := concat('#', @gml:id) return sort(root(.)//diggs:RIColumnConstruction[diggs:samplingFeatureRef/@xlink:href = $id]/diggs:installationRecord//diggs:timeDomain//(gml:timePosition | gml:endPosition | diggs:end))[last()]</t>
+          <t>let $id := concat('#', @gml:id), $a := (root(.)//diggs:RIColumnConstruction[diggs:samplingFeatureRef/@xlink:href = $id][.//diggs:TimeIntervalList[@unit = 'second']])[1] return if (exists($a)) then xs:dateTime($a/diggs:activityDateTime//diggs:start) + xs:dayTimeDuration(concat('PT', tokenize(normalize-space($a//diggs:TimeIntervalList/diggs:timeIntervalList), '\s+')[last()], 'S')) else ()</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>diggs:whenConstructed//diggs:end</t>
+          <t>let $id := concat('#', @gml:id) return sort(root(.)//diggs:RIColumnConstruction[diggs:samplingFeatureRef/@xlink:href = $id]/diggs:installationRecord//diggs:timeDomain//(gml:timePosition | gml:endPosition | diggs:end))[last()]</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3533,27 +3533,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>sampling_frequency</t>
+          <t>discharge_time</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>diggs:GroutBatch</t>
+          <t>diggs:RIColumn</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>frequency</t>
+          <t>difference</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>distinct-values($evidence//diggs:GroutSpecimen/diggs:extractionTime/normalize-space(.))</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>diggs:totalBatchVolume</t>
+          <t>diggs:whenConstructed//diggs:end</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>(diggs:samplingDate | diggs:deref(diggs:samplingActivityRef)/diggs:samplingDate)/diggs:TimeInterval/diggs:start</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>evidence</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3584,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>distinct-values(for $s in $evidence//diggs:GroutSpecimen[diggs:ageAtTest[@uom='d']] return string(xs:date(substring(string($s/ancestor::diggs:MaterialTest/diggs:samplingTime//gml:timePosition), 1, 10)) - xs:dayTimeDuration(concat('P', $s/diggs:ageAtTest, 'D'))))</t>
+          <t>distinct-values($evidence//diggs:GroutSpecimen/diggs:extractionTime/normalize-space(.))</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3595,32 +3600,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>penetration_over_interval</t>
+          <t>sampling_frequency</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>diggs:RIColumn</t>
+          <t>diggs:GroutBatch</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>change_over_window</t>
+          <t>frequency</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>diggs:series(($evidence/descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth')</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>let $s := diggs:series((descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth'), $m := max($s ! ?2) return ($s[?2 = $m])[1]?1</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>evidence</t>
+          <t>distinct-values(for $s in $evidence//diggs:GroutSpecimen[diggs:ageAtTest[@uom='d']] return string(xs:date(substring(string($s/ancestor::diggs:MaterialTest/diggs:samplingTime//gml:timePosition), 1, 10)) - xs:dayTimeDuration(concat('P', $s/diggs:ageAtTest, 'D'))))</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>diggs:totalBatchVolume</t>
         </is>
       </c>
     </row>
@@ -3628,6 +3628,36 @@
       <c r="A29">
         <f>IF(ISNA(VLOOKUP(B29,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>penetration_over_interval</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>diggs:RIColumn</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>change_over_window</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>diggs:series(($evidence/descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth')</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>let $s := diggs:series((descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth'), $m := max($s ! ?2) return ($s[?2 = $m])[1]?1</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
RCON1: discharge_time - binding for a TimePositionList record domain
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1867,7 +1867,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>The time elapsed from the introduction of mixing water to the end of discharge of the mix at the point of placement - a limit on how long a grout or concrete batch may take to be placed. Evaluated on the element that received the batch: the end of its installation record where one exists (the activity start plus the last elapsed time of a time-interval-list domain, or the last time of an instant domain), otherwise the end of its whenConstructed interval, less the start of the batch's sampling (mixing) activity. The two times must be recorded to a resolution at least as fine as the unit of the limit (hours need a time of day; days need only a date); otherwise the value is not evaluable.</t>
+          <t>The time elapsed from the introduction of mixing water to the end of discharge of the mix at the point of placement - a limit on how long a grout or concrete batch may take to be placed. Evaluated on the element that received the batch: the end of its installation record where one exists (the activity start plus the last elapsed time of a time-interval-list domain, the last time of a time-position-list domain, or the last time of an instant domain), otherwise the end of its whenConstructed interval, less the start of the batch's sampling (mixing) activity. The two times must be recorded to a resolution at least as fine as the unit of the limit (hours need a time of day; days need only a date); otherwise the value is not evaluable.</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>let $id := concat('#', @gml:id) return sort(root(.)//diggs:RIColumnConstruction[diggs:samplingFeatureRef/@xlink:href = $id]/diggs:installationRecord//diggs:timeDomain//(gml:timePosition | gml:endPosition | diggs:end))[last()]</t>
+          <t>let $id := concat('#', @gml:id), $a := (root(.)//diggs:RIColumnConstruction[diggs:samplingFeatureRef/@xlink:href = $id][.//diggs:TimePositionList])[1] return if (exists($a)) then tokenize(normalize-space($a//diggs:TimePositionList/diggs:timePositionList), '\s+')[last()] else ()</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3548,7 +3548,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>diggs:whenConstructed//diggs:end</t>
+          <t>let $id := concat('#', @gml:id) return sort(root(.)//diggs:RIColumnConstruction[diggs:samplingFeatureRef/@xlink:href = $id]/diggs:installationRecord//diggs:timeDomain//(gml:timePosition | gml:endPosition | diggs:end))[last()]</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3569,27 +3569,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>sampling_frequency</t>
+          <t>discharge_time</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>diggs:GroutBatch</t>
+          <t>diggs:RIColumn</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>frequency</t>
+          <t>difference</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>distinct-values($evidence//diggs:GroutSpecimen/diggs:extractionTime/normalize-space(.))</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>diggs:totalBatchVolume</t>
+          <t>diggs:whenConstructed//diggs:end</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>(diggs:samplingDate | diggs:deref(diggs:samplingActivityRef)/diggs:samplingDate)/diggs:TimeInterval/diggs:start</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>evidence</t>
         </is>
       </c>
     </row>
@@ -3615,7 +3620,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>distinct-values(for $s in $evidence//diggs:GroutSpecimen[diggs:ageAtTest[@uom='d']] return string(xs:date(substring(string($s/ancestor::diggs:MaterialTest/diggs:samplingTime//gml:timePosition), 1, 10)) - xs:dayTimeDuration(concat('P', $s/diggs:ageAtTest, 'D'))))</t>
+          <t>distinct-values($evidence//diggs:GroutSpecimen/diggs:extractionTime/normalize-space(.))</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3631,32 +3636,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>penetration_over_interval</t>
+          <t>sampling_frequency</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>diggs:RIColumn</t>
+          <t>diggs:GroutBatch</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>change_over_window</t>
+          <t>frequency</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>diggs:series(($evidence/descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth')</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>let $s := diggs:series((descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth'), $m := max($s ! ?2) return ($s[?2 = $m])[1]?1</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>evidence</t>
+          <t>distinct-values(for $s in $evidence//diggs:GroutSpecimen[diggs:ageAtTest[@uom='d']] return string(xs:date(substring(string($s/ancestor::diggs:MaterialTest/diggs:samplingTime//gml:timePosition), 1, 10)) - xs:dayTimeDuration(concat('P', $s/diggs:ageAtTest, 'D'))))</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>diggs:totalBatchVolume</t>
         </is>
       </c>
     </row>
@@ -3664,6 +3664,36 @@
       <c r="A30">
         <f>IF(ISNA(VLOOKUP(B30,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>penetration_over_interval</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>diggs:RIColumn</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>change_over_window</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>diggs:series(($evidence/descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth')</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>let $s := diggs:series((descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth'), $m := max($s ! ?2) return ($s[?2 = $m])[1]?1</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
CAD2: cuttingToolType dictionary; recordingParameter occurrences in mwd_properties and gr_inj_properties; installation-record conditions for depth and hydraulic_torque_pressure; penetration_over_interval judged on the construction activity (referenceSource subject)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1831,7 +1831,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>The distance the installation tool advances into the ground over a stated interval of time - for example less than 50 mm over two consecutive minutes as a drilling refusal rule. The interval is stated by an evidenceCondition (interval_duration) on the criterion. Distinct from penetration_rate, which is the same advance expressed per unit time. Evaluated on the installation record: the depth gained over the window of that duration that ends when the tool first reaches its maximum depth, so a refusal rule judges the last push before termination and not the pause at total depth. Depth is positive downward.</t>
+          <t>The distance the installation tool advances into the ground over a stated interval of time - for example less than 50 mm over two consecutive minutes as a drilling refusal rule. The interval is stated by an evidenceCondition (interval_duration) on the criterion. Distinct from penetration_rate, which is the same advance expressed per unit time. Evaluated on the construction activity that formed the element, from its installation record: the depth gained over the window of that duration that ends when the tool first reaches its maximum depth, so a refusal rule judges the last push before termination and not the pause at total depth. Depth is positive downward.</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>diggs:RIColumn</t>
+          <t>diggs:RIColumnConstruction</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3682,7 +3682,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>diggs:series(($evidence/descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth')</t>
+          <t>diggs:series((descendant-or-self::diggs:RIInstallationRecord[.//diggs:propertyClass/@codeSpace[ends-with(., '#depth')]])[1], 'depth')</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3692,7 +3692,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>evidence</t>
+          <t>subject</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PLT2: designProperty maximum_test_stress (minimum stress a load test must reach), bound to the procedure's maxTestStress
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1927,12 +1927,36 @@
         <f>IF(ISNA(VLOOKUP(B28,AssociatedElements!B$2:B2966,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B28" s="13" t="n"/>
-      <c r="C28" s="13" t="n"/>
-      <c r="D28" s="14" t="n"/>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="13" t="n"/>
-      <c r="G28" s="9" t="n"/>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>maximum_test_stress</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>Maximum test stress</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>The highest stress a load test is taken to - the largest stress applied through the bearing plate or loaded footprint during the test. A requirement on how the test is run, stated as a minimum the test must reach (for example 150 % of the design bearing pressure). Compared with the maxTestStress of the test's procedure.</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>pressure</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2">
@@ -2634,7 +2658,21 @@
         <f>IF(ISNA(VLOOKUP(B28,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B28" s="13" t="n"/>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>maximum_test_stress</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -3700,6 +3738,21 @@
       <c r="A31">
         <f>IF(ISNA(VLOOKUP(B31,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>maximum_test_stress</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>diggs:procedure/*/diggs:maxTestStress</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PLT3: designProperty load_increment_count, increment_hold_duration, settlement_change_last_five_minutes, bound to the load-test increments
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1963,36 +1963,104 @@
         <f>IF(ISNA(VLOOKUP(B29,AssociatedElements!B$2:B2967,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B29" s="13" t="n"/>
-      <c r="C29" s="13" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="13" t="n"/>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>load_increment_count</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Load increment count</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>The number of loading increments applied in a load test - the stages in which load was raised, not the unloading stages. A requirement on how the test is run, stated as a minimum (for example at least three increments). Counted from the increments of the test's procedure.</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
       <c r="F29" s="13" t="n"/>
-      <c r="G29" s="9" t="n"/>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2">
         <f>IF(ISNA(VLOOKUP(B30,AssociatedElements!B$2:B2968,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B30" s="13" t="n"/>
-      <c r="C30" s="13" t="n"/>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="13" t="n"/>
-      <c r="G30" s="9" t="n"/>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>increment_hold_duration</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Load increment hold duration</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>The time a load increment is held before the next is applied, taken from the first to the last reading of the increment, in seconds. One value for each loading increment of the test; the criterion's statistic states which governs (the shortest, for a minimum hold). A requirement on how the test is run.</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2">
         <f>IF(ISNA(VLOOKUP(B31,AssociatedElements!B$2:B2969,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B31" s="13" t="n"/>
-      <c r="C31" s="18" t="n"/>
-      <c r="D31" s="19" t="n"/>
-      <c r="E31" s="18" t="n"/>
-      <c r="F31" s="18" t="n"/>
-      <c r="G31" s="9" t="n"/>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>settlement_change_last_five_minutes</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>Settlement change over the last five minutes of an increment</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>The settlement gained over the last five minutes of a load increment's hold - the settlement at the last reading minus the settlement five minutes earlier, interpolated. One value for each loading increment of the test; the criterion's statistic states which governs (the largest, for a stabilization requirement). A requirement on how the test is run, for example that an increment is held until the settlement in five minutes is less than 0.02 mm.</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F31" s="18" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2">
@@ -2679,21 +2747,63 @@
         <f>IF(ISNA(VLOOKUP(B29,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B29" s="13" t="n"/>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>load_increment_count</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
         <f>IF(ISNA(VLOOKUP(B30,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B30" s="13" t="n"/>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>increment_hold_duration</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
         <f>IF(ISNA(VLOOKUP(B31,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B31" s="13" t="n"/>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>settlement_change_last_five_minutes</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -2819,7 +2929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3752,6 +3862,57 @@
       <c r="E31" t="inlineStr">
         <is>
           <t>diggs:procedure/*/diggs:maxTestStress</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>load_increment_count</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>count(diggs:procedure/*/diggs:increment/diggs:LoadTestIncrement[diggs:loadingPhase = 'loading'])</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>increment_hold_duration</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>for $i in diggs:procedure/*/diggs:increment/diggs:LoadTestIncrement[diggs:loadingPhase = 'loading'] return (diggs:series($i//diggs:TemporalResult, 'settlement'))[last()]?1</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>settlement_change_last_five_minutes</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>for $i in diggs:procedure/*/diggs:increment/diggs:LoadTestIncrement[diggs:loadingPhase = 'loading'] return let $s := diggs:series($i//diggs:TemporalResult, 'settlement'), $e := ($s[last()])?1 return diggs:valueAt($s, $e) - diggs:valueAt($s, $e - 300)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PIT2: designProperty test_count and averaged_impact_count; properties toe_depth, toe_depth_deviation and relative_reflection_amplitude for low-strain integrity test criteria
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -2067,24 +2067,64 @@
         <f>IF(ISNA(VLOOKUP(B32,AssociatedElements!B$2:B2970,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B32" s="13" t="n"/>
-      <c r="C32" s="18" t="n"/>
-      <c r="D32" s="19" t="n"/>
-      <c r="E32" s="18" t="n"/>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>test_count</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>Test count</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>The number of tests made under a planned measurement - for example the number of integrity tests made of a planned set of locations. A requirement on how much testing is done, stated as a minimum. Counted from the realized measurements that cite the planned measurement.</t>
+        </is>
+      </c>
+      <c r="E32" s="18" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
       <c r="F32" s="18" t="n"/>
-      <c r="G32" s="9" t="n"/>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2">
         <f>IF(ISNA(VLOOKUP(B33,AssociatedElements!B$2:B2971,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B33" s="13" t="n"/>
-      <c r="C33" s="18" t="n"/>
-      <c r="D33" s="19" t="n"/>
-      <c r="E33" s="18" t="n"/>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>averaged_impact_count</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>Averaged impact count</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>The number of hammer impacts averaged into one record of a low-strain integrity test, as reported by the test equipment. A requirement on how the test is run, stated as a minimum (for example at least three). One value for each test.</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
       <c r="F33" s="18" t="n"/>
-      <c r="G33" s="9" t="n"/>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2">
@@ -2810,14 +2850,42 @@
         <f>IF(ISNA(VLOOKUP(B32,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B32" s="13" t="n"/>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>test_count</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
         <f>IF(ISNA(VLOOKUP(B33,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B33" s="13" t="n"/>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>averaged_impact_count</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34">

</xml_diff>

<commit_message>
PIT2: designProperty age_at_test and strength_at_test; lowStrainTestMethod retired (testMethod is now an enumeration in the schema)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -2131,24 +2131,72 @@
         <f>IF(ISNA(VLOOKUP(B34,AssociatedElements!B$2:B2972,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="18" t="n"/>
-      <c r="D34" s="19" t="n"/>
-      <c r="E34" s="18" t="n"/>
-      <c r="F34" s="18" t="n"/>
-      <c r="G34" s="9" t="n"/>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>age_at_test</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>Age at test</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>The age of an element when a test is made on it: the time from the end of its construction to the start of the test. A requirement on when a test may be made, stated as a minimum - for example seven days for a low strain integrity test of a cast-in-place pile.</t>
+        </is>
+      </c>
+      <c r="E34" s="18" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F34" s="18" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2">
         <f>IF(ISNA(VLOOKUP(B35,AssociatedElements!B$2:B2973,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B35" s="13" t="n"/>
-      <c r="C35" s="18" t="n"/>
-      <c r="D35" s="19" t="n"/>
-      <c r="E35" s="18" t="n"/>
-      <c r="F35" s="18" t="n"/>
-      <c r="G35" s="9" t="n"/>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>strength_at_test</t>
+        </is>
+      </c>
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>Strength at test</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>The compressive strength of the concrete of an element at the age of a test made on it, as a percentage of its design strength. A requirement on when a test may be made, stated as a minimum - for example 75 percent for a low strain integrity test of a cast-in-place pile. Evaluated from compressive strength tests of the concrete made no later than the test: where none was made by then the strength at test is not known and the requirement is not shown to be met.</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F35" s="18" t="inlineStr">
+        <is>
+          <t>dimensionless</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2">
@@ -2892,14 +2940,42 @@
         <f>IF(ISNA(VLOOKUP(B34,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B34" s="13" t="n"/>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>age_at_test</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
         <f>IF(ISNA(VLOOKUP(B35,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B35" s="13" t="n"/>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>strength_at_test</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:DesignConformanceCriterion</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36">

</xml_diff>

<commit_message>
PIT4: value bindings for the low strain test criteria (test_count, averaged_impact_count, age_at_test, strength_at_test, position on a Test; toe_depth_deviation, relative_reflection_amplitude, relative_toe_amplitude); relative_toe_amplitude (property and evidence condition: the balanced-record band); verificationOutcome inconclusive
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -3073,7 +3073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4057,6 +4057,116 @@
       <c r="E34" t="inlineStr">
         <is>
           <t>for $i in diggs:procedure/*/diggs:increment/diggs:LoadTestIncrement[diggs:loadingPhase = 'loading'] return let $s := diggs:series($i//diggs:TemporalResult, 'settlement'), $e := ($s[last()])?1 return diggs:valueAt($s, $e) - diggs:valueAt($s, $e - 300)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>test_count</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>diggs:Test</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>count(root(.)//diggs:Test[diggs:programDesignRef/@xlink:href = concat('#', $design/@gml:id)])</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>averaged_impact_count</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>diggs:Test</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>diggs:procedure/*/diggs:averagedImpactCount</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>age_at_test</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>diggs:Test</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>days-from-duration(xs:date(substring(string(diggs:samplingTime//gml:timePosition), 1, 10)) - xs:date(substring(string(diggs:deref(diggs:samplingFeatureRef)/diggs:whenConstructed//diggs:end), 1, 10)))</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>strength_at_test</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>diggs:Test</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>let $col := diggs:deref(diggs:samplingFeatureRef), $batch := $col/diggs:groutRef/@xlink:href, $d := xs:date(substring(string(diggs:samplingTime//gml:timePosition), 1, 10)), $mix := diggs:deref(diggs:deref(diggs:deref($col/diggs:groutRef)/diggs:samplingActivityRef)/diggs:currentDesign//diggs:programDesignRef), $r := (for $m in root(.)//diggs:MaterialTest[diggs:sampleRef/@xlink:href = $batch][xs:date(substring(string(diggs:samplingTime//gml:timePosition), 1, 10)) le $d] return diggs:series($m/diggs:outcome/*, 'compressive_strength_unconfined') ! ?2) return if (exists($r) and exists($mix/diggs:strengthDesign)) then max($r) * 1000000 div number($mix/diggs:strengthDesign) * 100 else ()</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>diggs:Test</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>if (exists(diggs:realizesGridIndex) and exists($design//diggs:ReferenceableGridByArray)) then (let $n := tokenize(normalize-space(($design//diggs:ReferenceableGridByArray)[1]/gml:posList), '\s+'), $i := number(normalize-space(diggs:realizesGridIndex)), $p := tokenize(normalize-space(diggs:deref(diggs:samplingFeatureRef)/diggs:referencePoint//gml:pos), '\s+') return math:sqrt(math:pow(number($p[1]) - number($n[2*$i + 1]), 2) + math:pow(number($p[2]) - number($n[2*$i + 2]), 2))) else ()</t>
         </is>
       </c>
     </row>

</xml_diff>